<commit_message>
Add BB2 cuttlet plots and BB3 cuttlet data programs and deliverables
- skills/bb2_cuttlet_plots.py: generates cuttlet cross-section plots per assembly
- skills/bb3_cuttlet_data.py: extracts centroid X, Y, area per cuttlet to Excel
- Assy_2176r06 deliverables: plot image + data file (32 cuttlets, 0.9742 in²)
- Master tracker updated to 3/6 linked for 2176r06

https://claude.ai/code/session_01N8TFjZHRi9fPjGEUiAzPPF
</commit_message>
<xml_diff>
--- a/assemblies/master_tracker.xlsx
+++ b/assemblies/master_tracker.xlsx
@@ -530,14 +530,14 @@
           <t>Source File</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Cuttlet Plots</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Cuttlet Data</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -562,6 +562,8 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>